<commit_message>
Add gitignore for Excel temp files
</commit_message>
<xml_diff>
--- a/dataset/Sample_dataset.xlsx
+++ b/dataset/Sample_dataset.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Micropump_flowrate_optimization\dataset\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8C9EB6-1336-4696-9A68-6DE88E4DB9D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,22 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="3">
+  <si>
+    <t>Ts(sec)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Pc(bars)</t>
+  </si>
+  <si>
+    <t>Flowrate(g(m)L/min)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -29,12 +49,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +75,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +357,622 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:O13"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C2" s="1">
+        <v>-2E-3</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F2" s="1">
+        <v>-8.0000000000000002E-3</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I2" s="1">
+        <v>-8.7999999999999995E-2</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L2" s="1">
+        <v>-4.0000000000000001E-3</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O2" s="1">
+        <v>4.3920000000000003</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1.2E-2</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0.16200000000000001</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I3" s="1">
+        <v>5.274</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L3" s="1">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O3" s="1">
+        <v>4.75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1.2E-2</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0.14599999999999999</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I4" s="1">
+        <v>6.9139999999999997</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L4" s="1">
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O4" s="1">
+        <v>3.266</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.124</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I5" s="1">
+        <v>5.9459999999999997</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N5" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O5" s="1">
+        <v>4.2939999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0.222</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0.152</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I6" s="1">
+        <v>5.0359999999999996</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L6" s="1">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N6" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O6" s="1">
+        <v>4.5739999999999998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B7" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0.154</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F7" s="1">
+        <v>0.69</v>
+      </c>
+      <c r="G7" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I7" s="1">
+        <v>4.6920000000000002</v>
+      </c>
+      <c r="J7" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K7" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L7" s="1">
+        <v>1.0780000000000001</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O7" s="1">
+        <v>4.508</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B8" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0.14399999999999999</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F8" s="1">
+        <v>1.6020000000000001</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I8" s="1">
+        <v>4.2220000000000004</v>
+      </c>
+      <c r="J8" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K8" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L8" s="1">
+        <v>2.2559999999999998</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N8" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O8" s="1">
+        <v>4.2619999999999996</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B9" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C9" s="1">
+        <v>0.17199999999999999</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F9" s="1">
+        <v>3.1920000000000002</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H9" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I9" s="1">
+        <v>4.0179999999999998</v>
+      </c>
+      <c r="J9" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K9" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L9" s="1">
+        <v>0.71599999999999997</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N9" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O9" s="1">
+        <v>4.5780000000000003</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B10" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0.48599999999999999</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F10" s="1">
+        <v>5.6020000000000003</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I10" s="1">
+        <v>3.8660000000000001</v>
+      </c>
+      <c r="J10" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K10" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L10" s="1">
+        <v>0.10199999999999999</v>
+      </c>
+      <c r="M10" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N10" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O10" s="1">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1.31</v>
+      </c>
+      <c r="D11" s="1">
+        <v>1</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F11" s="1">
+        <v>8</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I11" s="1">
+        <v>3.8820000000000001</v>
+      </c>
+      <c r="J11" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L11" s="1">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="M11" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N11" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O11" s="1">
+        <v>3.7879999999999998</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B12" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C12" s="1">
+        <v>3.1160000000000001</v>
+      </c>
+      <c r="D12" s="1">
+        <v>1</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F12" s="1">
+        <v>8</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H12" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I12" s="1">
+        <v>6.516</v>
+      </c>
+      <c r="J12" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L12" s="1">
+        <v>3.5999999999999997E-2</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N12" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O12" s="1">
+        <v>4.3499999999999996</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>1.5</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="C13" s="1">
+        <v>5.0880000000000001</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="F13" s="1">
+        <v>8</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="I13" s="1">
+        <v>7.87</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0.25</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="L13" s="1">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0.125</v>
+      </c>
+      <c r="N13" s="1">
+        <v>0.03</v>
+      </c>
+      <c r="O13" s="1">
+        <v>4.3079999999999998</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>